<commit_message>
feat: deliver reports only in PDF format on email and update verified records
</commit_message>
<xml_diff>
--- a/reports/2026-10-16/private_scholarships_report_2026-10-16.xlsx
+++ b/reports/2026-10-16/private_scholarships_report_2026-10-16.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Report Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Active Opportunities'!$A$1:$R$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Priority Highlights'!$A$1:$R$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Active Opportunities'!$A$1:$R$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Priority Highlights'!$A$1:$R$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'International'!$A$1:$R$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Watchlist (Awaiting Call)'!$A$1:$R$2</definedName>
   </definedNames>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -691,13 +691,1058 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0018</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>75th Celebration of Independence Day of Pakistan Scholarship Program</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Government of Pakistan</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>federal govt</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>world's top 25 ranked universities</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>MS and PhD</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>world's top 25 ranked universities</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>https://eportal.hec.gov.pk/idps75</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hec.gov.pk/english/scholarshipsgrants/IDPS/Pages/default.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0008</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CM Foreign Scholarship</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Khyber Pakhtunkhwa Education Foundation (KPEF)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>provincial govt</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/scholarship/cm_foreign_scholarship</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0017</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Chief Minister Foreign Scholarship Program</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Chief Minister of Khyber Pakhtunkhwa through Khyber Pakhtunkhwa Education Foundation</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>provincial govt</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>selected universities in the People's Republic of China</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Language &amp; Culture, BS, MS, and PhD Programs</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>merit cum in-affordability basis</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/scholarship/cm_foreign_scholarship</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0009</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>KP Youth Scholarship</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Khyber Pakhtunkhwa Education Foundation (KPEF)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>provincial govt</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>HE Government Colleges in Khyber Pakhtunkhwa</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>good academic merit</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/scholarship/youth_scholarship</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>HEC Need Based Scholarships</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Higher Education Commission, Islamabad / Government of Pakistan</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>federal govt</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>participating public sector Universities/Institutions and their campuses which are receiving annual recurring grant through Higher Education Commission, Islamabad</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>talented students</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hec.gov.pk/english/scholarshipsgrants/NBS/Pages/default.aspx</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hec.gov.pk/english/scholarshipsgrants/NBS/Pages/default.aspx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R2"/>
+  <autoFilter ref="A1:R7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="35" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="35" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opportunity Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sponsor Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Days Left</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Charsadda Eligible</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>KP Domicile</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Target Uni</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Award Amount</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Eligible Institutions</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Degree Levels</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Merit Criteria</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Need / Income Cap</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Apply URL</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0003</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Abasyn University Peshawar Merit &amp; Need-Based Scholarship</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Abasyn University Peshawar</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>university</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>25% to 100% tuition fee discount</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Abasyn University Peshawar Campus</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Undergraduate, Master's</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Above 3.00 CGPA or 70% marks for merit scholarships</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>PKR 60,000 per month</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>https://abasyn.edu.pk/scholarships/apply</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>https://abasyn.edu.pk/scholarships/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0018</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>75th Celebration of Independence Day of Pakistan Scholarship Program</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Government of Pakistan</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>federal govt</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>world's top 25 ranked universities</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>MS and PhD</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>world's top 25 ranked universities</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>https://eportal.hec.gov.pk/idps75</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hec.gov.pk/english/scholarshipsgrants/IDPS/Pages/default.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0008</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CM Foreign Scholarship</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Khyber Pakhtunkhwa Education Foundation (KPEF)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>provincial govt</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/scholarship/cm_foreign_scholarship</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0017</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Chief Minister Foreign Scholarship Program</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Chief Minister of Khyber Pakhtunkhwa through Khyber Pakhtunkhwa Education Foundation</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>provincial govt</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>selected universities in the People's Republic of China</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Language &amp; Culture, BS, MS, and PhD Programs</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>merit cum in-affordability basis</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/scholarship/cm_foreign_scholarship</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SCH-202610-0009</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>KP Youth Scholarship</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Khyber Pakhtunkhwa Education Foundation (KPEF)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>provincial govt</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>HE Government Colleges in Khyber Pakhtunkhwa</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>good academic merit</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/scholarship/youth_scholarship</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>https://ef.kp.gov.pk/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:R6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -821,36 +1866,38 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SCH-202610-0003</t>
+          <t>SCH-202610-0016</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Abasyn University Peshawar Merit &amp; Need-Based Scholarship</t>
+          <t>Commonwealth Scholarship Programme (Master’s &amp; PhD)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Abasyn University Peshawar</t>
+          <t>Commonwealth / Higher Education Commission Pakistan</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>university</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>international</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Deadline not stated</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>30</v>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
@@ -869,32 +1916,32 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>25% to 100% tuition fee discount</t>
+          <t>not stated</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Abasyn University Peshawar Campus</t>
+          <t>not stated</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Undergraduate, Master's</t>
+          <t>Master’s &amp; PhD</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Above 3.00 CGPA or 70% marks for merit scholarships</t>
+          <t>HEC accepts valid test score of HAT</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>PKR 60,000 per month</t>
+          <t>not stated</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>https://abasyn.edu.pk/scholarships/apply</t>
+          <t>https://www.hec.gov.pk/english/HECAnnouncements/Pages/CW-Scholarship.aspx</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
@@ -904,134 +1951,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>https://abasyn.edu.pk/scholarships/</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:R2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="35" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="35" customWidth="1" min="18" max="18"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Opportunity Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Sponsor Type</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Days Left</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Charsadda Eligible</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>KP Domicile</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Target Uni</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Award Amount</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Eligible Institutions</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Degree Levels</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Merit Criteria</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Need / Income Cap</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Apply URL</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Verification</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Source URL</t>
+          <t>https://www.hec.gov.pk/english/scholarshipsgrants/lao/Pages/default.aspx</t>
         </is>
       </c>
     </row>
@@ -1213,7 +2133,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-16 09:14 PKT</t>
+          <t>2026-10-16 19:42 PKT</t>
         </is>
       </c>
     </row>
@@ -1225,7 +2145,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RUN-20261016-091400</t>
+          <t>RUN-20261016-194227</t>
         </is>
       </c>
     </row>
@@ -1246,7 +2166,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -1256,7 +2176,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -1276,7 +2196,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1286,7 +2206,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
chore: add reports and state update for 2026-10-17
</commit_message>
<xml_diff>
--- a/reports/2026-10-16/private_scholarships_report_2026-10-16.xlsx
+++ b/reports/2026-10-16/private_scholarships_report_2026-10-16.xlsx
@@ -2133,7 +2133,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-16 19:42 PKT</t>
+          <t>2026-10-16 19:53 PKT</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RUN-20261016-194227</t>
+          <t>RUN-20261016-195337</t>
         </is>
       </c>
     </row>

</xml_diff>